<commit_message>
Add spatial mapping and refactor flow-salinity plots
Integrate sf package for geospatial analysis with Florida outline shapefile. Refactor ggplot_hyperbolic_fit() to support plotting all models simultaneously using patchwork, with improved error handling for failed fits. Update station map to use spatial features and remove debug statement.
</commit_message>
<xml_diff>
--- a/PBC/Data/F5595_Stations.xlsx
+++ b/PBC/Data/F5595_Stations.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Erica.Williams\Documents\GitHub\Oyster-Reports\PBC\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Erica.Williams\Documents\GitHub\Oyster-Reports\PBC\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{C0184416-16A7-45EE-9840-FB19B1BECCD4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2D3B4519-5863-4923-B107-E48B2D24BA23}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28740" yWindow="105" windowWidth="21600" windowHeight="11235" xr2:uid="{27411A20-8021-4061-B973-66ABA9E50B4C}"/>
+    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{27411A20-8021-4061-B973-66ABA9E50B4C}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -473,9 +473,9 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2CB3CA53-1649-4C60-8B25-B2592EF58D88}">
   <dimension ref="A1:D12"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -489,7 +489,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>4</v>
       </c>
@@ -503,7 +503,7 @@
         <v>26.669683333333332</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>4</v>
       </c>
@@ -517,7 +517,7 @@
         <v>26.647466666666666</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>4</v>
       </c>
@@ -531,7 +531,7 @@
         <v>26.597516666666667</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>4</v>
       </c>
@@ -545,7 +545,7 @@
         <v>26.632566666666666</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>4</v>
       </c>
@@ -559,7 +559,7 @@
         <v>26.623999999999999</v>
       </c>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>4</v>
       </c>
@@ -573,7 +573,7 @@
         <v>26.687633333333334</v>
       </c>
     </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>16</v>
       </c>
@@ -581,13 +581,13 @@
         <v>11</v>
       </c>
       <c r="C8">
-        <v>-80.203344999999999</v>
+        <v>-80.055209000000005</v>
       </c>
       <c r="D8">
-        <v>26.679839000000001</v>
-      </c>
-    </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
+        <v>26.644667999999999</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>16</v>
       </c>
@@ -601,7 +601,7 @@
         <v>26.539110999999998</v>
       </c>
     </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>16</v>
       </c>
@@ -615,7 +615,7 @@
         <v>26.817226999999999</v>
       </c>
     </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>16</v>
       </c>
@@ -629,7 +629,7 @@
         <v>26.675305999999999</v>
       </c>
     </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>16</v>
       </c>

</xml_diff>